<commit_message>
Efectivo y Equivalentes: arreglo de consola + módulo (arquitectura, E1–E4 backend, E7 vista de 3 pasos) (#193)
Arreglo de la colisión de CSS de la consola-chat + inicio del módulo de Efectivo y Equivalentes por etapas: documento de arquitectura con el inventario de 17 botones; E1 validaciones cruzadas de ingesta y moneda; E2 motor de reproceso por niveles N1-N7 con reconstrucción y comparación vs la compañía; E3 matriz del reproceso por cuenta y endpoint; E4 prescripción parametrizable, partidas duplicadas y recurrentes; E7 vista de 3 pasos (tema oscuro) solo para Efectivo. Verificado con pytest y vitest/build.
</commit_message>
<xml_diff>
--- a/frontend/public/ejemplos/efectivo_equivalentes/RQ-001_cuentas.xlsx
+++ b/frontend/public/ejemplos/efectivo_equivalentes/RQ-001_cuentas.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,50 +435,55 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Moneda</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Saldo según libros</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Saldo según estado bancario (o arqueo en caja)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Saldo confirmado por el banco</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Restringido (Sí/No)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Monto restringido</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Motivo de la restricción</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Fin de la restricción</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Restringido ya presentado aparte (Sí/No)</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Fecha de adquisición (inversiones)</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Fecha de vencimiento (inversiones)</t>
         </is>
@@ -502,15 +507,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>500.00</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>500.00</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
@@ -518,6 +527,7 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -537,15 +547,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>300.00</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>300.00</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
@@ -553,6 +567,7 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -572,26 +587,31 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>125680.50</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>131210.50</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>131210.50</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -611,46 +631,51 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>47700.00</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>45900.00</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>45900.00</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>10000.00</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Garantía de préstamo (pignoración)</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>30/06/2027</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -670,26 +695,31 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>22000.00</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>22000.00</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>21500.00</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -709,38 +739,43 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>1650.00</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>1200.00</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
         <is>
           <t>Sí</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>1650.00</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Embargo judicial</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -760,26 +795,31 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
           <t>-3200.00</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>-3200.00</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>-3200.00</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -799,30 +839,35 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
           <t>50000.00</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>50000.00</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>50000.00</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr">
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
         <is>
           <t>15/11/2025</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>14/01/2026</t>
         </is>
@@ -846,30 +891,35 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
           <t>30000.00</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>30000.00</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>30000.00</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr">
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
         <is>
           <t>01/10/2025</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>30/03/2026</t>
         </is>

</xml_diff>